<commit_message>
memoria-resumo v3: HBM supply by vendor (UBS Fig 3x8) + NAND/house sufficiency; theme page wired
General UBS tie-out (Memory Semis 03-jul-26): band A/D anchors match Fig 33 (rev 151/692/1,248, suff -2.3/-8.1/-1.2, ASP 0.48/1.78/2.69) and Fig 41 NAND. New in band C: HBM bit supply by vendor = Fig 3 supply x Fig 8 share - Hynix 12.7->17.5->23.0 bn Gb (59->48->39%), Samsung 4.3->11.0->24.2 (20->30->41%, OVERTAKES in 27E), Micron 4.5->7.7->11.8. New in band D: NAND sufficiency (Fig 41: -1.0/-9.3/-0.7%) replacing the wrong 'no S/D series' note, and house model-based DRAM sufficiency (-1.3/-8.8/+2.6% - the 2027 flip vs UBS -1.2%). hbm-memory theme page: dashboards pointer block + Sources entry + changelog. Extract now also pulls hbm_ubs/nand_suff/dram_suff_house from the bible; 89 rows.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_wiki/_dashboards/memoria-resumo.xlsx
+++ b/_wiki/_dashboards/memoria-resumo.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_dados" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'RESUMO'!$A$1:$I$84</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'RESUMO'!$A$1:$I$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -318,37 +318,52 @@
         <t>Se o handset NÃO tivesse cortado: 26E ≈ −10,7% (vs −8,1%) e 27E ≈ −3,7% (vs −1,2%). Denominadores: 386,7 = 358,3 bn Gb ex-HBM (engine, aba capacidade) + 28,4 HBM (build); 520,1 = 474,5 + 45,6 — base engine, ~2% abaixo da soma das linhas da banda B (bases UBS ligeiramente distintas). A destruição de demanda é o amortecedor que o bear case subestima.</t>
       </text>
     </comment>
-    <comment ref="A52" authorId="0" shapeId="0">
+    <comment ref="A45" authorId="0" shapeId="0">
+      <text>
+        <t>Oferta UBS 59,1 bn Gb 27E vs demanda house 45,6 (units Capstone abaixo da street) e vs Redburn 50 revisado por alocação — a folga é o debate. Share Fig 8: Hynix 59→48→39%, Samsung 20→30→41% (ULTRAPASSA em 27E), Micron ~21/21/20%.</t>
+      </text>
+    </comment>
+    <comment ref="A56" authorId="0" shapeId="0">
       <text>
         <t>O aperto que o blended esconde: −14,6% em 27E. Vira ≈0 em 28E porque a demanda de wafers HBM flatten (~695k) e os adds novos vão p/ DDR.</t>
       </text>
     </comment>
-    <comment ref="A56" authorId="0" shapeId="0">
+    <comment ref="A57" authorId="0" shapeId="0">
+      <text>
+        <t>O DEBATE de 2027: com as NOSSAS units de IA (abaixo da street), 2026 segue ~−9% mas 2027 FLIPA para ~+3% equilibrado — vs UBS −1,2%. O 28E house é a visão do engine de wafers (≈0), não desta linha.</t>
+      </text>
+    </comment>
+    <comment ref="A58" authorId="0" shapeId="0">
+      <text>
+        <t>Supply 995/1.172/1.410 vs demanda inv-adj 1.005/1.293/1.419 bn GB → −1,0%/−9,3%/−0,7%. ASP $/GB 0,07→0,26→0,37 (+5,5× do vale). Mesma forma da DRAM: aperto máximo em 26E.</t>
+      </text>
+    </comment>
+    <comment ref="A61" authorId="0" shapeId="0">
       <text>
         <t>Caem 1.535→1.486 até 27E mesmo com capex recorde — tudo que entra é absorvido pelo HBM. 28E: 1.786 (a virada).</t>
       </text>
     </comment>
-    <comment ref="A58" authorId="0" shapeId="0">
+    <comment ref="A63" authorId="0" shapeId="0">
       <text>
         <t>Cada wafer migrado p/ HBM entrega ~1/3 dos bits (TSV/stacking/yield). Melhora ~25%/ano de densidade HBM (HBM4 12-16Hi).</t>
       </text>
     </comment>
-    <comment ref="A59" authorId="0" shapeId="0">
+    <comment ref="A64" authorId="0" shapeId="0">
       <text>
         <t>129 bn Gb em 27E = 24% da demanda — maior que o crescimento da própria demanda; driver #1 do preço de DDR.</t>
       </text>
     </comment>
-    <comment ref="A71" authorId="0" shapeId="0">
+    <comment ref="A76" authorId="0" shapeId="0">
       <text>
         <t>Sockets recalibrados = CPUs Bernstein ÷ servidores UBS (1,5-2,0×; o 2S flat superestimava ~25%). Bernstein: 31,8 / 51,6 / 61,6M em 25/27/28E, incl. Grace 6,1M (27E) sem DIMM.</t>
       </text>
     </comment>
-    <comment ref="A74" authorId="0" shapeId="0">
+    <comment ref="A79" authorId="0" shapeId="0">
       <text>
         <t>46→66 GB (25→27E) — cruza com mix 64→96/128GB RDIMM. MRDIMM = 12% do mix em 28E (Bernstein).</t>
       </text>
     </comment>
-    <comment ref="A75" authorId="0" shapeId="0">
+    <comment ref="A80" authorId="0" shapeId="0">
       <text>
         <t>Redburn: NVDA HBM ~$17-18/GB 2026 → $30-32/GB 2027 (+70-80%); JPM/Micron: blended +~30%. O build fica entre os dois.</t>
       </text>
@@ -647,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2009,53 +2024,75 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>HBM — capacidade por fornecedor</t>
-        </is>
-      </c>
-      <c r="B42" s="19" t="inlineStr">
-        <is>
-          <t>k wpm 26E: Samsung 689 UBS / 740 TF · SK Hynix 609 / 610 · Micron 317 / 365  —  27E UBS: 737 / 671 / 357</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="n"/>
-      <c r="D42" s="9" t="n"/>
-      <c r="E42" s="9" t="n"/>
-      <c r="F42" s="9" t="n"/>
-      <c r="G42" s="9" t="n"/>
-      <c r="H42" s="9" t="n"/>
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>HBM — SK Hynix</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>bn Gb</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="21" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="F42" s="21" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G42" s="21" t="n">
+        <v>23</v>
+      </c>
+      <c r="H42" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>UBS vs TrendForce</t>
+          <t>UBS Fig 3 × Fig 8 (03-jul)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>NAND — Samsung</t>
+          <t>HBM — Samsung</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>bn GB</t>
-        </is>
-      </c>
-      <c r="C43" s="21" t="n">
-        <v>254.1842295</v>
-      </c>
-      <c r="D43" s="21" t="n">
-        <v>296.67056581</v>
+          <t>bn Gb</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="E43" s="21" t="n">
-        <v>305.67011685</v>
+        <v>4.3</v>
       </c>
       <c r="F43" s="21" t="n">
-        <v>347.88733109</v>
+        <v>11</v>
       </c>
       <c r="G43" s="21" t="n">
-        <v>405.81331861</v>
+        <v>24.2</v>
       </c>
       <c r="H43" s="15" t="inlineStr">
         <is>
@@ -2064,35 +2101,39 @@
       </c>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>UBS Fig 3 × Fig 8 (03-jul)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>NAND — Kioxia</t>
+          <t>HBM — Micron</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>bn GB</t>
-        </is>
-      </c>
-      <c r="C44" s="21" t="n">
-        <v>105.82072995</v>
-      </c>
-      <c r="D44" s="21" t="n">
-        <v>130.475883</v>
+          <t>bn Gb</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="E44" s="21" t="n">
-        <v>148.05620765</v>
+        <v>4.5</v>
       </c>
       <c r="F44" s="21" t="n">
-        <v>173.85671617</v>
+        <v>7.7</v>
       </c>
       <c r="G44" s="21" t="n">
-        <v>211.10658193</v>
+        <v>11.8</v>
       </c>
       <c r="H44" s="15" t="inlineStr">
         <is>
@@ -2101,35 +2142,39 @@
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>UBS Fig 3 × Fig 8 (03-jul)</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="14" t="inlineStr">
-        <is>
-          <t>NAND — SanDisk</t>
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>HBM — total oferta (UBS)</t>
         </is>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>bn GB</t>
-        </is>
-      </c>
-      <c r="C45" s="21" t="n">
-        <v>100.91351069</v>
-      </c>
-      <c r="D45" s="21" t="n">
-        <v>101.29813451</v>
-      </c>
-      <c r="E45" s="21" t="n">
-        <v>119.22047837</v>
-      </c>
-      <c r="F45" s="21" t="n">
-        <v>139.43212069</v>
-      </c>
-      <c r="G45" s="21" t="n">
-        <v>162.97394192</v>
+          <t>bn Gb</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" s="20" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="F45" s="20" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="G45" s="20" t="n">
+        <v>59.1</v>
       </c>
       <c r="H45" s="15" t="inlineStr">
         <is>
@@ -2138,51 +2183,37 @@
       </c>
       <c r="I45" s="13" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>UBS Fig 3</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="14" t="inlineStr">
-        <is>
-          <t>NAND — SK Hynix</t>
-        </is>
-      </c>
-      <c r="B46" s="11" t="inlineStr">
-        <is>
-          <t>bn GB</t>
-        </is>
-      </c>
-      <c r="C46" s="21" t="n">
-        <v>148.50344718</v>
-      </c>
-      <c r="D46" s="21" t="n">
-        <v>143.57220984</v>
-      </c>
-      <c r="E46" s="21" t="n">
-        <v>160.56266612</v>
-      </c>
-      <c r="F46" s="21" t="n">
-        <v>192.3809966</v>
-      </c>
-      <c r="G46" s="21" t="n">
-        <v>233.67540086</v>
-      </c>
-      <c r="H46" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    share HBM (Fig 8)</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="inlineStr">
+        <is>
+          <t>Hynix 59% → 48% → 39% · Samsung 20% → 30% → 41% (ultrapassa em 27E) · Micron 21% → 21% → 20% — capacidade k wpm 26E: Samsung 689 UBS / 740 TF · SK 609/610 · MU 317/365</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="n"/>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="F46" s="9" t="n"/>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="9" t="n"/>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>UBS Fig 8 · TrendForce</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>NAND — Micron</t>
+          <t>NAND — Samsung</t>
         </is>
       </c>
       <c r="B47" s="11" t="inlineStr">
@@ -2191,19 +2222,19 @@
         </is>
       </c>
       <c r="C47" s="21" t="n">
-        <v>90.02957563000001</v>
+        <v>254.1842295</v>
       </c>
       <c r="D47" s="21" t="n">
-        <v>106.60903975</v>
+        <v>296.67056581</v>
       </c>
       <c r="E47" s="21" t="n">
-        <v>133.88101337</v>
+        <v>305.67011685</v>
       </c>
       <c r="F47" s="21" t="n">
-        <v>161.21827732</v>
+        <v>347.88733109</v>
       </c>
       <c r="G47" s="21" t="n">
-        <v>188.92000809</v>
+        <v>405.81331861</v>
       </c>
       <c r="H47" s="15" t="inlineStr">
         <is>
@@ -2219,238 +2250,286 @@
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
         <is>
+          <t>NAND — Kioxia</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>bn GB</t>
+        </is>
+      </c>
+      <c r="C48" s="21" t="n">
+        <v>105.82072995</v>
+      </c>
+      <c r="D48" s="21" t="n">
+        <v>130.475883</v>
+      </c>
+      <c r="E48" s="21" t="n">
+        <v>148.05620765</v>
+      </c>
+      <c r="F48" s="21" t="n">
+        <v>173.85671617</v>
+      </c>
+      <c r="G48" s="21" t="n">
+        <v>211.10658193</v>
+      </c>
+      <c r="H48" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>NAND — SanDisk</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>bn GB</t>
+        </is>
+      </c>
+      <c r="C49" s="21" t="n">
+        <v>100.91351069</v>
+      </c>
+      <c r="D49" s="21" t="n">
+        <v>101.29813451</v>
+      </c>
+      <c r="E49" s="21" t="n">
+        <v>119.22047837</v>
+      </c>
+      <c r="F49" s="21" t="n">
+        <v>139.43212069</v>
+      </c>
+      <c r="G49" s="21" t="n">
+        <v>162.97394192</v>
+      </c>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I49" s="13" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>NAND — SK Hynix</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>bn GB</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="n">
+        <v>148.50344718</v>
+      </c>
+      <c r="D50" s="21" t="n">
+        <v>143.57220984</v>
+      </c>
+      <c r="E50" s="21" t="n">
+        <v>160.56266612</v>
+      </c>
+      <c r="F50" s="21" t="n">
+        <v>192.3809966</v>
+      </c>
+      <c r="G50" s="21" t="n">
+        <v>233.67540086</v>
+      </c>
+      <c r="H50" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>NAND — Micron</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>bn GB</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="n">
+        <v>90.02957563000001</v>
+      </c>
+      <c r="D51" s="21" t="n">
+        <v>106.60903975</v>
+      </c>
+      <c r="E51" s="21" t="n">
+        <v>133.88101337</v>
+      </c>
+      <c r="F51" s="21" t="n">
+        <v>161.21827732</v>
+      </c>
+      <c r="G51" s="21" t="n">
+        <v>188.92000809</v>
+      </c>
+      <c r="H51" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
           <t>NAND — YMTC</t>
         </is>
       </c>
-      <c r="B48" s="11" t="inlineStr">
+      <c r="B52" s="11" t="inlineStr">
         <is>
           <t>bn GB</t>
         </is>
       </c>
-      <c r="C48" s="21" t="n">
+      <c r="C52" s="21" t="n">
         <v>41.82680343</v>
       </c>
-      <c r="D48" s="21" t="n">
+      <c r="D52" s="21" t="n">
         <v>75.74131974999999</v>
       </c>
-      <c r="E48" s="21" t="n">
+      <c r="E52" s="21" t="n">
         <v>119.13197936</v>
       </c>
-      <c r="F48" s="21" t="n">
+      <c r="F52" s="21" t="n">
         <v>148.33805253</v>
       </c>
-      <c r="G48" s="21" t="n">
+      <c r="G52" s="21" t="n">
         <v>197.47627264</v>
       </c>
-      <c r="H48" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I48" s="13" t="inlineStr">
+      <c r="H52" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I52" s="13" t="inlineStr">
         <is>
           <t>UBS</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>NAND — total oferta</t>
-        </is>
-      </c>
-      <c r="B49" s="11" t="inlineStr">
-        <is>
-          <t>bn GB</t>
-        </is>
-      </c>
-      <c r="C49" s="20" t="n">
-        <v>748.35829638</v>
-      </c>
-      <c r="D49" s="20" t="n">
-        <v>862.08715266</v>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>994.88246172</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>1172.1134944</v>
-      </c>
-      <c r="G49" s="20" t="n">
-        <v>1409.60552405</v>
-      </c>
-      <c r="H49" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I49" s="13" t="inlineStr">
-        <is>
-          <t>UBS</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>D · SUFICIÊNCIA (S/D − 1) — a síntese</t>
-        </is>
-      </c>
-      <c r="B50" s="9" t="n"/>
-      <c r="C50" s="9" t="n"/>
-      <c r="D50" s="9" t="n"/>
-      <c r="E50" s="9" t="n"/>
-      <c r="F50" s="9" t="n"/>
-      <c r="G50" s="9" t="n"/>
-      <c r="H50" s="9" t="n"/>
-      <c r="I50" s="9" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="10" t="inlineStr">
-        <is>
-          <t>DRAM blended</t>
-        </is>
-      </c>
-      <c r="B51" s="11" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C51" s="24" t="n">
-        <v>-0.0036</v>
-      </c>
-      <c r="D51" s="24" t="n">
-        <v>-0.0233</v>
-      </c>
-      <c r="E51" s="24" t="n">
-        <v>-0.0235</v>
-      </c>
-      <c r="F51" s="24" t="n">
-        <v>-0.0813</v>
-      </c>
-      <c r="G51" s="24" t="n">
-        <v>-0.012</v>
-      </c>
-      <c r="H51" s="15" t="inlineStr">
-        <is>
-          <t>≈0 eng.</t>
-        </is>
-      </c>
-      <c r="I51" s="13" t="inlineStr">
-        <is>
-          <t>UBS · engine</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="10" t="inlineStr">
-        <is>
-          <t>DDR ex-HBM</t>
-        </is>
-      </c>
-      <c r="B52" s="11" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C52" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D52" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E52" s="24" t="n">
-        <v>-0.0433</v>
-      </c>
-      <c r="F52" s="24" t="n">
-        <v>-0.0156</v>
-      </c>
-      <c r="G52" s="24" t="n">
-        <v>-0.1461</v>
-      </c>
-      <c r="H52" s="24" t="n">
-        <v>-0.0032</v>
-      </c>
-      <c r="I52" s="13" t="inlineStr">
-        <is>
-          <t>engine house</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>HBM</t>
-        </is>
-      </c>
-      <c r="B53" s="19" t="inlineStr">
-        <is>
-          <t>sold out CY26 incl. HBM4 (Micron Q1 FY26) · 27E oferta revisada 60→50 bn Gb-equiv por alocação, não demanda</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="n"/>
-      <c r="D53" s="9" t="n"/>
-      <c r="E53" s="9" t="n"/>
-      <c r="F53" s="9" t="n"/>
-      <c r="G53" s="9" t="n"/>
-      <c r="H53" s="9" t="n"/>
+          <t>NAND — total oferta</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>bn GB</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="n">
+        <v>748.35829638</v>
+      </c>
+      <c r="D53" s="20" t="n">
+        <v>862.08715266</v>
+      </c>
+      <c r="E53" s="20" t="n">
+        <v>994.88246172</v>
+      </c>
+      <c r="F53" s="20" t="n">
+        <v>1172.1134944</v>
+      </c>
+      <c r="G53" s="20" t="n">
+        <v>1409.60552405</v>
+      </c>
+      <c r="H53" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="I53" s="13" t="inlineStr">
         <is>
-          <t>assumptions ledger</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
-        <is>
-          <t>NAND</t>
-        </is>
-      </c>
-      <c r="B54" s="19" t="inlineStr">
-        <is>
-          <t>sem série S/D no modelo — proxy: ASP $/GB 0,066 → 0,256 → 0,33-0,37 (25→27E, +5,5× do vale)</t>
-        </is>
-      </c>
+          <t>UBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>D · SUFICIÊNCIA (S/D − 1) — a síntese</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="n"/>
       <c r="C54" s="9" t="n"/>
       <c r="D54" s="9" t="n"/>
       <c r="E54" s="9" t="n"/>
       <c r="F54" s="9" t="n"/>
       <c r="G54" s="9" t="n"/>
       <c r="H54" s="9" t="n"/>
-      <c r="I54" s="13" t="inlineStr">
-        <is>
-          <t>UBS · cenários</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="15" customHeight="1">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>E · CAPACIDADE, CANIBALIZAÇÃO HBM E CAPEX</t>
-        </is>
-      </c>
-      <c r="B55" s="9" t="n"/>
-      <c r="C55" s="9" t="n"/>
-      <c r="D55" s="9" t="n"/>
-      <c r="E55" s="9" t="n"/>
-      <c r="F55" s="9" t="n"/>
-      <c r="G55" s="9" t="n"/>
-      <c r="H55" s="9" t="n"/>
-      <c r="I55" s="9" t="n"/>
+      <c r="I54" s="9" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>DRAM blended</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C55" s="24" t="n">
+        <v>-0.0036</v>
+      </c>
+      <c r="D55" s="24" t="n">
+        <v>-0.0233</v>
+      </c>
+      <c r="E55" s="24" t="n">
+        <v>-0.0235</v>
+      </c>
+      <c r="F55" s="24" t="n">
+        <v>-0.0813</v>
+      </c>
+      <c r="G55" s="24" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="H55" s="15" t="inlineStr">
+        <is>
+          <t>≈0 eng.</t>
+        </is>
+      </c>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>UBS · engine</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="14" t="inlineStr">
-        <is>
-          <t>Wafers DDR</t>
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>DDR ex-HBM</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>k wpm</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
@@ -2463,33 +2542,33 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E56" s="16" t="n">
-        <v>1535</v>
-      </c>
-      <c r="F56" s="16" t="n">
-        <v>1498</v>
-      </c>
-      <c r="G56" s="16" t="n">
-        <v>1486</v>
-      </c>
-      <c r="H56" s="16" t="n">
-        <v>1785.5</v>
+      <c r="E56" s="24" t="n">
+        <v>-0.0433</v>
+      </c>
+      <c r="F56" s="24" t="n">
+        <v>-0.0156</v>
+      </c>
+      <c r="G56" s="24" t="n">
+        <v>-0.1461</v>
+      </c>
+      <c r="H56" s="24" t="n">
+        <v>-0.0032</v>
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>engine (Fig.9 UBS)</t>
+          <t>engine house</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="14" t="inlineStr">
-        <is>
-          <t>Wafers HBM</t>
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>DRAM blended — HOUSE (units Capstone, inv-adj)</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>k wpm</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C57" s="15" t="inlineStr">
@@ -2502,33 +2581,35 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E57" s="16" t="n">
-        <v>390</v>
-      </c>
-      <c r="F57" s="16" t="n">
-        <v>500</v>
-      </c>
-      <c r="G57" s="16" t="n">
-        <v>690</v>
-      </c>
-      <c r="H57" s="16" t="n">
-        <v>694.5</v>
+      <c r="E57" s="24" t="n">
+        <v>-0.0131</v>
+      </c>
+      <c r="F57" s="24" t="n">
+        <v>-0.0881</v>
+      </c>
+      <c r="G57" s="24" t="n">
+        <v>0.0262</v>
+      </c>
+      <c r="H57" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>SemiAnalysis · engine</t>
+          <t>bíblia Memory S&amp;D (modelo)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>Penalidade de wafer HBM (bits DDR ÷ bits HBM por wafer)</t>
+          <t>NAND (S/D−1)</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>%</t>
         </is>
       </c>
       <c r="C58" s="15" t="inlineStr">
@@ -2541,708 +2622,740 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E58" s="25" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F58" s="25" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="G58" s="25" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="H58" s="25" t="n">
-        <v>3.1</v>
+      <c r="E58" s="17" t="n">
+        <v>-0.0101</v>
+      </c>
+      <c r="F58" s="17" t="n">
+        <v>-0.0935</v>
+      </c>
+      <c r="G58" s="17" t="n">
+        <v>-0.0066</v>
+      </c>
+      <c r="H58" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>engine</t>
+          <t>UBS Fig.41</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
+          <t>HBM</t>
+        </is>
+      </c>
+      <c r="B59" s="19" t="inlineStr">
+        <is>
+          <t>sold out CY26 incl. HBM4 (Micron Q1 FY26) · 27E oferta revisada 60→50 bn Gb-equiv por alocação, não demanda · oferta UBS por vendor na banda C</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="n"/>
+      <c r="D59" s="9" t="n"/>
+      <c r="E59" s="9" t="n"/>
+      <c r="F59" s="9" t="n"/>
+      <c r="G59" s="9" t="n"/>
+      <c r="H59" s="9" t="n"/>
+      <c r="I59" s="13" t="inlineStr">
+        <is>
+          <t>assumptions ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15" customHeight="1">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>E · CAPACIDADE, CANIBALIZAÇÃO HBM E CAPEX</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="n"/>
+      <c r="C60" s="9" t="n"/>
+      <c r="D60" s="9" t="n"/>
+      <c r="E60" s="9" t="n"/>
+      <c r="F60" s="9" t="n"/>
+      <c r="G60" s="9" t="n"/>
+      <c r="H60" s="9" t="n"/>
+      <c r="I60" s="9" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>Wafers DDR</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>k wpm</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="n">
+        <v>1535</v>
+      </c>
+      <c r="F61" s="16" t="n">
+        <v>1498</v>
+      </c>
+      <c r="G61" s="16" t="n">
+        <v>1486</v>
+      </c>
+      <c r="H61" s="16" t="n">
+        <v>1785.5</v>
+      </c>
+      <c r="I61" s="13" t="inlineStr">
+        <is>
+          <t>engine (Fig.9 UBS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>Wafers HBM</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>k wpm</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="n">
+        <v>390</v>
+      </c>
+      <c r="F62" s="16" t="n">
+        <v>500</v>
+      </c>
+      <c r="G62" s="16" t="n">
+        <v>690</v>
+      </c>
+      <c r="H62" s="16" t="n">
+        <v>694.5</v>
+      </c>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
+          <t>SemiAnalysis · engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>Penalidade de wafer HBM (bits DDR ÷ bits HBM por wafer)</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="25" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F63" s="25" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G63" s="25" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H63" s="25" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="inlineStr">
+        <is>
           <t>Bits líquidos perdidos p/ HBM (% da demanda)</t>
         </is>
       </c>
-      <c r="B59" s="11" t="inlineStr">
+      <c r="B64" s="11" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C59" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D59" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E59" s="24" t="n">
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="24" t="n">
         <v>0.1646</v>
       </c>
-      <c r="F59" s="24" t="n">
+      <c r="F64" s="24" t="n">
         <v>0.2042</v>
       </c>
-      <c r="G59" s="24" t="n">
+      <c r="G64" s="24" t="n">
         <v>0.2415</v>
       </c>
-      <c r="H59" s="24" t="n">
+      <c r="H64" s="24" t="n">
         <v>0.2323</v>
       </c>
-      <c r="I59" s="13" t="inlineStr">
+      <c r="I64" s="13" t="inlineStr">
         <is>
           <t>engine</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="14" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
         <is>
           <t>Capex memória</t>
         </is>
       </c>
-      <c r="B60" s="11" t="inlineStr">
+      <c r="B65" s="11" t="inlineStr">
         <is>
           <t>$bn</t>
         </is>
       </c>
-      <c r="C60" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D60" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" s="16" t="n">
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="n">
         <v>75</v>
       </c>
-      <c r="F60" s="16" t="n">
+      <c r="F65" s="16" t="n">
         <v>85</v>
       </c>
-      <c r="G60" s="16" t="n">
+      <c r="G65" s="16" t="n">
         <v>120</v>
       </c>
-      <c r="H60" s="16" t="n">
+      <c r="H65" s="16" t="n">
         <v>140</v>
       </c>
-      <c r="I60" s="13" t="inlineStr">
+      <c r="I65" s="13" t="inlineStr">
         <is>
           <t>UBS · bridge</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="10" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t>Conta do capex (26E→27E)</t>
         </is>
       </c>
-      <c r="B61" s="19" t="inlineStr">
+      <c r="B66" s="19" t="inlineStr">
         <is>
           <t>greenfield/net-add 17→32 · conversão HBM+packaging 20→30 · node/manutenção 48→58 $bn</t>
         </is>
       </c>
-      <c r="C61" s="9" t="n"/>
-      <c r="D61" s="9" t="n"/>
-      <c r="E61" s="9" t="n"/>
-      <c r="F61" s="9" t="n"/>
-      <c r="G61" s="9" t="n"/>
-      <c r="H61" s="9" t="n"/>
-      <c r="I61" s="13" t="inlineStr">
+      <c r="C66" s="9" t="n"/>
+      <c r="D66" s="9" t="n"/>
+      <c r="E66" s="9" t="n"/>
+      <c r="F66" s="9" t="n"/>
+      <c r="G66" s="9" t="n"/>
+      <c r="H66" s="9" t="n"/>
+      <c r="I66" s="13" t="inlineStr">
         <is>
           <t>bíblia (ponte)</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="15" customHeight="1">
-      <c r="A62" s="8" t="inlineStr">
+    <row r="67" ht="15" customHeight="1">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>F · P&amp;L 27E POR EMPRESA → P/E (muda com o cenário ASP)</t>
         </is>
       </c>
-      <c r="B62" s="9" t="n"/>
-      <c r="C62" s="9" t="n"/>
-      <c r="D62" s="9" t="n"/>
-      <c r="E62" s="9" t="n"/>
-      <c r="F62" s="9" t="n"/>
-      <c r="G62" s="9" t="n"/>
-      <c r="H62" s="9" t="n"/>
-      <c r="I62" s="9" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="B67" s="9" t="n"/>
+      <c r="C67" s="9" t="n"/>
+      <c r="D67" s="9" t="n"/>
+      <c r="E67" s="9" t="n"/>
+      <c r="F67" s="9" t="n"/>
+      <c r="G67" s="9" t="n"/>
+      <c r="H67" s="9" t="n"/>
+      <c r="I67" s="9" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>vendor →</t>
         </is>
       </c>
-      <c r="B63" s="9" t="n"/>
-      <c r="C63" s="6" t="inlineStr">
+      <c r="B68" s="9" t="n"/>
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>Micron</t>
         </is>
       </c>
-      <c r="D63" s="6" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>SK Hynix</t>
         </is>
       </c>
-      <c r="E63" s="6" t="inlineStr">
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>Samsung*</t>
         </is>
       </c>
-      <c r="F63" s="6" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <t>Kioxia</t>
         </is>
       </c>
-      <c r="G63" s="6" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>SanDisk</t>
         </is>
       </c>
-      <c r="H63" s="9" t="n"/>
-      <c r="I63" s="13" t="inlineStr">
+      <c r="H68" s="9" t="n"/>
+      <c r="I68" s="13" t="inlineStr">
         <is>
           <t>BBG 02-jul · bíblia SxD</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="14" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
         <is>
           <t>Receita memória 27E (bits × ASP cenário)</t>
         </is>
       </c>
-      <c r="B64" s="11" t="inlineStr">
+      <c r="B69" s="11" t="inlineStr">
         <is>
           <t>$bn</t>
         </is>
       </c>
-      <c r="C64" s="16">
+      <c r="C69" s="16">
         <f>(_dados!B7*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C7*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))/1000</f>
         <v/>
       </c>
-      <c r="D64" s="16">
+      <c r="D69" s="16">
         <f>(_dados!B8*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C8*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))/1000</f>
         <v/>
       </c>
-      <c r="E64" s="16">
+      <c r="E69" s="16">
         <f>(_dados!B9*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C9*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))/1000</f>
         <v/>
       </c>
-      <c r="F64" s="16">
+      <c r="F69" s="16">
         <f>(_dados!B10*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C10*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))/1000</f>
         <v/>
       </c>
-      <c r="G64" s="16">
+      <c r="G69" s="16">
         <f>(_dados!B11*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C11*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))/1000</f>
         <v/>
       </c>
-      <c r="H64" s="9" t="n"/>
-      <c r="I64" s="13" t="inlineStr">
+      <c r="H69" s="9" t="n"/>
+      <c r="I69" s="13" t="inlineStr">
         <is>
           <t>fórmula = dashboard P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="14" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
         <is>
           <t>EPS 27E house (modelo)</t>
         </is>
       </c>
-      <c r="B65" s="11" t="inlineStr">
+      <c r="B70" s="11" t="inlineStr">
         <is>
           <t>local</t>
         </is>
       </c>
-      <c r="C65" s="16">
+      <c r="C70" s="16">
         <f>((_dados!B7*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C7*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))*_dados!D7-_dados!E7)*(1-_dados!F7)*_dados!G7/_dados!H7</f>
         <v/>
       </c>
-      <c r="D65" s="16">
+      <c r="D70" s="16">
         <f>((_dados!B8*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C8*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))*_dados!D8-_dados!E8)*(1-_dados!F8)*_dados!G8/_dados!H8</f>
         <v/>
       </c>
-      <c r="E65" s="16">
+      <c r="E70" s="16">
         <f>((_dados!B9*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C9*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))*_dados!D9-_dados!E9)*(1-_dados!F9)*_dados!G9/_dados!H9</f>
         <v/>
       </c>
-      <c r="F65" s="16">
+      <c r="F70" s="16">
         <f>((_dados!B10*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C10*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))*_dados!D10-_dados!E10)*(1-_dados!F10)*_dados!G10/_dados!H10</f>
         <v/>
       </c>
-      <c r="G65" s="16">
+      <c r="G70" s="16">
         <f>((_dados!B11*INDEX(_dados!$B$2:$B$4,MATCH($C$2,_dados!$A$2:$A$4,0))+_dados!C11*INDEX(_dados!$C$2:$C$4,MATCH($C$2,_dados!$A$2:$A$4,0)))*_dados!D11-_dados!E11)*(1-_dados!F11)*_dados!G11/_dados!H11</f>
         <v/>
       </c>
-      <c r="H65" s="9" t="n"/>
-      <c r="I65" s="13" t="inlineStr">
+      <c r="H70" s="9" t="n"/>
+      <c r="I70" s="13" t="inlineStr">
         <is>
           <t>gm×rev−opex, ×(1−tax)×fx÷ações</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="14" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
         <is>
           <t>P/E house @ px atual</t>
         </is>
       </c>
-      <c r="B66" s="11" t="inlineStr">
+      <c r="B71" s="11" t="inlineStr">
         <is>
           <t>×</t>
         </is>
       </c>
-      <c r="C66" s="25">
-        <f>_dados!I7/C65</f>
+      <c r="C71" s="25">
+        <f>_dados!I7/C70</f>
         <v/>
       </c>
-      <c r="D66" s="25">
-        <f>_dados!I8/D65</f>
+      <c r="D71" s="25">
+        <f>_dados!I8/D70</f>
         <v/>
       </c>
-      <c r="E66" s="25">
-        <f>_dados!I9/E65</f>
+      <c r="E71" s="25">
+        <f>_dados!I9/E70</f>
         <v/>
       </c>
-      <c r="F66" s="25">
-        <f>_dados!I10/F65</f>
+      <c r="F71" s="25">
+        <f>_dados!I10/F70</f>
         <v/>
       </c>
-      <c r="G66" s="25">
-        <f>_dados!I11/G65</f>
+      <c r="G71" s="25">
+        <f>_dados!I11/G70</f>
         <v/>
       </c>
-      <c r="H66" s="9" t="n"/>
-      <c r="I66" s="13" t="inlineStr">
+      <c r="H71" s="9" t="n"/>
+      <c r="I71" s="13" t="inlineStr">
         <is>
           <t>px BBG ÷ EPS modelo</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="10" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
         <is>
           <t>P/E consenso 27E (BBG)</t>
         </is>
       </c>
-      <c r="B67" s="11" t="inlineStr">
+      <c r="B72" s="11" t="inlineStr">
         <is>
           <t>×</t>
         </is>
       </c>
-      <c r="C67" s="26">
+      <c r="C72" s="26">
         <f>_dados!I7/_dados!J7</f>
         <v/>
       </c>
-      <c r="D67" s="26">
+      <c r="D72" s="26">
         <f>_dados!I8/_dados!J8</f>
         <v/>
       </c>
-      <c r="E67" s="26">
+      <c r="E72" s="26">
         <f>_dados!I9/_dados!J9</f>
         <v/>
       </c>
-      <c r="F67" s="26">
+      <c r="F72" s="26">
         <f>_dados!I10/_dados!J10</f>
         <v/>
       </c>
-      <c r="G67" s="26">
+      <c r="G72" s="26">
         <f>_dados!I11/_dados!J11</f>
         <v/>
       </c>
-      <c r="H67" s="9" t="n"/>
-      <c r="I67" s="13" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="10" t="inlineStr">
+      <c r="H72" s="9" t="n"/>
+      <c r="I72" s="13" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
         <is>
           <t>Δ EPS house vs consenso (o edge)</t>
         </is>
       </c>
-      <c r="B68" s="11" t="inlineStr">
+      <c r="B73" s="11" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C68" s="27">
-        <f>C65/_dados!J7-1</f>
+      <c r="C73" s="27">
+        <f>C70/_dados!J7-1</f>
         <v/>
       </c>
-      <c r="D68" s="27">
-        <f>D65/_dados!J8-1</f>
+      <c r="D73" s="27">
+        <f>D70/_dados!J8-1</f>
         <v/>
       </c>
-      <c r="E68" s="27">
-        <f>E65/_dados!J9-1</f>
+      <c r="E73" s="27">
+        <f>E70/_dados!J9-1</f>
         <v/>
       </c>
-      <c r="F68" s="27">
-        <f>F65/_dados!J10-1</f>
+      <c r="F73" s="27">
+        <f>F70/_dados!J10-1</f>
         <v/>
       </c>
-      <c r="G68" s="27">
-        <f>G65/_dados!J11-1</f>
+      <c r="G73" s="27">
+        <f>G70/_dados!J11-1</f>
         <v/>
       </c>
-      <c r="H68" s="9" t="n"/>
-      <c r="I68" s="13" t="inlineStr">
+      <c r="H73" s="9" t="n"/>
+      <c r="I73" s="13" t="inlineStr">
         <is>
           <t>modelo ÷ BBG − 1</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="10" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="10" t="inlineStr">
         <is>
           <t>*Samsung</t>
         </is>
       </c>
-      <c r="B69" s="19" t="inlineStr">
+      <c r="B74" s="19" t="inlineStr">
         <is>
           <t>consenso = empresa inteira (foundry/mobile/display) — P/E consenso não é 1:1 com o P&amp;L memória-only. EPS local: MU/SNDK $, SK/Samsung ₩, Kioxia ¥.</t>
         </is>
       </c>
-      <c r="C69" s="9" t="n"/>
-      <c r="D69" s="9" t="n"/>
-      <c r="E69" s="9" t="n"/>
-      <c r="F69" s="9" t="n"/>
-      <c r="G69" s="9" t="n"/>
-      <c r="H69" s="9" t="n"/>
-      <c r="I69" s="13" t="inlineStr"/>
-    </row>
-    <row r="70" ht="15" customHeight="1">
-      <c r="A70" s="8" t="inlineStr">
+      <c r="C74" s="9" t="n"/>
+      <c r="D74" s="9" t="n"/>
+      <c r="E74" s="9" t="n"/>
+      <c r="F74" s="9" t="n"/>
+      <c r="G74" s="9" t="n"/>
+      <c r="H74" s="9" t="n"/>
+      <c r="I74" s="13" t="inlineStr"/>
+    </row>
+    <row r="75" ht="15" customHeight="1">
+      <c r="A75" s="8" t="inlineStr">
         <is>
           <t>G · BUILDS — CROSS-CHECKS BOTTOM-UP</t>
         </is>
       </c>
-      <c r="B70" s="9" t="n"/>
-      <c r="C70" s="9" t="n"/>
-      <c r="D70" s="9" t="n"/>
-      <c r="E70" s="9" t="n"/>
-      <c r="F70" s="9" t="n"/>
-      <c r="G70" s="9" t="n"/>
-      <c r="H70" s="9" t="n"/>
-      <c r="I70" s="9" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="14" t="inlineStr">
+      <c r="B75" s="9" t="n"/>
+      <c r="C75" s="9" t="n"/>
+      <c r="D75" s="9" t="n"/>
+      <c r="E75" s="9" t="n"/>
+      <c r="F75" s="9" t="n"/>
+      <c r="G75" s="9" t="n"/>
+      <c r="H75" s="9" t="n"/>
+      <c r="I75" s="9" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="inlineStr">
         <is>
           <t>CPUs de servidor</t>
         </is>
       </c>
-      <c r="B71" s="11" t="inlineStr">
+      <c r="B76" s="11" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C71" s="21" t="n">
+      <c r="C76" s="21" t="n">
         <v>22.6</v>
       </c>
-      <c r="D71" s="21" t="n">
+      <c r="D76" s="21" t="n">
         <v>24</v>
       </c>
-      <c r="E71" s="21" t="n">
+      <c r="E76" s="21" t="n">
         <v>32.2</v>
       </c>
-      <c r="F71" s="21" t="n">
+      <c r="F76" s="21" t="n">
         <v>40.6</v>
       </c>
-      <c r="G71" s="21" t="n">
+      <c r="G76" s="21" t="n">
         <v>52.8</v>
       </c>
-      <c r="H71" s="21" t="n">
+      <c r="H76" s="21" t="n">
         <v>61.2</v>
       </c>
-      <c r="I71" s="13" t="inlineStr">
+      <c r="I76" s="13" t="inlineStr">
         <is>
           <t>Bernstein/Mercury (recal.)</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="10" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
         <is>
           <t>DRAM convencional por CPU</t>
         </is>
       </c>
-      <c r="B72" s="11" t="inlineStr">
+      <c r="B77" s="11" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="C72" s="12" t="n">
+      <c r="C77" s="12" t="n">
         <v>314</v>
       </c>
-      <c r="D72" s="12" t="n">
+      <c r="D77" s="12" t="n">
         <v>340</v>
       </c>
-      <c r="E72" s="12" t="n">
+      <c r="E77" s="12" t="n">
         <v>393</v>
       </c>
-      <c r="F72" s="12" t="n">
+      <c r="F77" s="12" t="n">
         <v>475</v>
       </c>
-      <c r="G72" s="12" t="n">
+      <c r="G77" s="12" t="n">
         <v>590</v>
       </c>
-      <c r="H72" s="12" t="n">
+      <c r="H77" s="12" t="n">
         <v>683</v>
       </c>
-      <c r="I72" s="13" t="inlineStr">
+      <c r="I77" s="13" t="inlineStr">
         <is>
           <t>modelo (conv ÷ CPUs)</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="14" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
         <is>
           <t>DIMMs por CPU</t>
         </is>
       </c>
-      <c r="B73" s="11" t="inlineStr">
+      <c r="B78" s="11" t="inlineStr">
         <is>
           <t>un.</t>
         </is>
       </c>
-      <c r="C73" s="25" t="n">
+      <c r="C78" s="25" t="n">
         <v>7.9</v>
       </c>
-      <c r="D73" s="25" t="n">
+      <c r="D78" s="25" t="n">
         <v>8.9</v>
       </c>
-      <c r="E73" s="25" t="n">
+      <c r="E78" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="F73" s="25" t="n">
+      <c r="F78" s="25" t="n">
         <v>9.5</v>
       </c>
-      <c r="G73" s="25" t="n">
+      <c r="G78" s="25" t="n">
         <v>10.3</v>
       </c>
-      <c r="H73" s="25" t="n">
+      <c r="H78" s="25" t="n">
         <v>11.7</v>
       </c>
-      <c r="I73" s="13" t="inlineStr">
+      <c r="I78" s="13" t="inlineStr">
         <is>
           <t>Bernstein (canais×slots×ocup.)</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="14" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
         <is>
           <t>GB por DIMM implícito</t>
         </is>
       </c>
-      <c r="B74" s="11" t="inlineStr">
+      <c r="B79" s="11" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="C74" s="16" t="n">
+      <c r="C79" s="16" t="n">
         <v>39</v>
       </c>
-      <c r="D74" s="16" t="n">
+      <c r="D79" s="16" t="n">
         <v>38</v>
       </c>
-      <c r="E74" s="16" t="n">
+      <c r="E79" s="16" t="n">
         <v>46</v>
       </c>
-      <c r="F74" s="16" t="n">
+      <c r="F79" s="16" t="n">
         <v>54</v>
       </c>
-      <c r="G74" s="16" t="n">
+      <c r="G79" s="16" t="n">
         <v>66</v>
       </c>
-      <c r="H74" s="16" t="n">
+      <c r="H79" s="16" t="n">
         <v>65</v>
       </c>
-      <c r="I74" s="13" t="inlineStr">
+      <c r="I79" s="13" t="inlineStr">
         <is>
           <t>modelo ÷ DIMMs Bernstein</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="14" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
         <is>
           <t>HBM $/GB blended (build)</t>
         </is>
       </c>
-      <c r="B75" s="11" t="inlineStr">
+      <c r="B80" s="11" t="inlineStr">
         <is>
           <t>$/GB</t>
         </is>
       </c>
-      <c r="C75" s="25" t="n">
+      <c r="C80" s="25" t="n">
         <v>10.5</v>
       </c>
-      <c r="D75" s="25" t="n">
+      <c r="D80" s="25" t="n">
         <v>14.6</v>
       </c>
-      <c r="E75" s="25" t="n">
+      <c r="E80" s="25" t="n">
         <v>16.7</v>
       </c>
-      <c r="F75" s="25" t="n">
+      <c r="F80" s="25" t="n">
         <v>17.9</v>
       </c>
-      <c r="G75" s="25" t="n">
+      <c r="G80" s="25" t="n">
         <v>21.3</v>
       </c>
-      <c r="H75" s="25" t="n">
+      <c r="H80" s="25" t="n">
         <v>25.9</v>
       </c>
-      <c r="I75" s="13" t="inlineStr">
+      <c r="I80" s="13" t="inlineStr">
         <is>
           <t>build (rev ÷ bits × 8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="10" t="inlineStr">
-        <is>
-          <t>HBM $/GB por geração</t>
-        </is>
-      </c>
-      <c r="B76" s="19" t="inlineStr">
-        <is>
-          <t>preço build: HBM3E $17 · HBM4 $26 · HBM4E $29 — mix bits: 26E 3E 84% / 4 13% → 27E 3E 51% / 4 46% → 28E 3E 14% / 4 45% / 4E 41%</t>
-        </is>
-      </c>
-      <c r="C76" s="9" t="n"/>
-      <c r="D76" s="9" t="n"/>
-      <c r="E76" s="9" t="n"/>
-      <c r="F76" s="9" t="n"/>
-      <c r="G76" s="9" t="n"/>
-      <c r="H76" s="9" t="n"/>
-      <c r="I76" s="13" t="inlineStr">
-        <is>
-          <t>build (por gen) · debate Redburn vs JPM</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="14" t="inlineStr">
-        <is>
-          <t>Smartphone GB/unidade</t>
-        </is>
-      </c>
-      <c r="B77" s="11" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="C77" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D77" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E77" s="25" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="F77" s="25" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="G77" s="25" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="H77" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I77" s="13" t="inlineStr">
-        <is>
-          <t>UBS Fig. (BOM 12→40%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="15" customHeight="1">
-      <c r="A78" s="8" t="inlineStr">
-        <is>
-          <t>H · DEBATES VIVOS, CATALISADORES E CONVENÇÕES</t>
-        </is>
-      </c>
-      <c r="B78" s="9" t="n"/>
-      <c r="C78" s="9" t="n"/>
-      <c r="D78" s="9" t="n"/>
-      <c r="E78" s="9" t="n"/>
-      <c r="F78" s="9" t="n"/>
-      <c r="G78" s="9" t="n"/>
-      <c r="H78" s="9" t="n"/>
-      <c r="I78" s="9" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="10" t="inlineStr">
-        <is>
-          <t>Virada 2028</t>
-        </is>
-      </c>
-      <c r="B79" s="19" t="inlineStr">
-        <is>
-          <t>house: déficit fecha ≈0 (wafers HBM flatten ~695k, adds vão p/ DDR) vs Bernstein +5% surplus — os 109,6 bn Gb de HBM deles em 28E exigiriam ~1,1M wafers e matariam o próprio surplus</t>
-        </is>
-      </c>
-      <c r="C79" s="9" t="n"/>
-      <c r="D79" s="9" t="n"/>
-      <c r="E79" s="9" t="n"/>
-      <c r="F79" s="9" t="n"/>
-      <c r="G79" s="9" t="n"/>
-      <c r="H79" s="9" t="n"/>
-      <c r="I79" s="13" t="inlineStr">
-        <is>
-          <t>engine · Bernstein SxD</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="10" t="inlineStr">
-        <is>
-          <t>Alocação 26</t>
-        </is>
-      </c>
-      <c r="B80" s="19" t="inlineStr">
-        <is>
-          <t>general-server DDR ultrapassou HBM como prioridade #1 de alocação (Redburn/TrendForce) — e ainda assim HBM sobe: $17-18 → $30-32/GB 27E (Redburn) vs blended +30% (JPM/Micron)</t>
-        </is>
-      </c>
-      <c r="C80" s="9" t="n"/>
-      <c r="D80" s="9" t="n"/>
-      <c r="E80" s="9" t="n"/>
-      <c r="F80" s="9" t="n"/>
-      <c r="G80" s="9" t="n"/>
-      <c r="H80" s="9" t="n"/>
-      <c r="I80" s="13" t="inlineStr">
-        <is>
-          <t>assumptions ledger</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>HBM $/GB por geração</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
         <is>
-          <t>CXMT: 4% da oferta DRAM 25 → 12% 27E (UBS) + IPO a caminho; YMTC 41→? bn GB NAND — o wildcard de oferta pós-28</t>
+          <t>preço build: HBM3E $17 · HBM4 $26 · HBM4E $29 — mix bits: 26E 3E 84% / 4 13% → 27E 3E 51% / 4 46% → 28E 3E 14% / 4 45% / 4E 41%</t>
         </is>
       </c>
       <c r="C81" s="9" t="n"/>
@@ -3253,65 +3366,75 @@
       <c r="H81" s="9" t="n"/>
       <c r="I81" s="13" t="inlineStr">
         <is>
-          <t>UBS · ledger</t>
+          <t>build (por gen) · debate Redburn vs JPM</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="10" t="inlineStr">
-        <is>
-          <t>Conteúdo</t>
-        </is>
-      </c>
-      <c r="B82" s="19" t="inlineStr">
-        <is>
-          <t>MRDIMM 12% do mix 28E (Bernstein) + 12/16-canais → DIMMs/CPU 9→11,7 — upside de conteúdo independente de units</t>
-        </is>
-      </c>
-      <c r="C82" s="9" t="n"/>
-      <c r="D82" s="9" t="n"/>
-      <c r="E82" s="9" t="n"/>
-      <c r="F82" s="9" t="n"/>
-      <c r="G82" s="9" t="n"/>
-      <c r="H82" s="9" t="n"/>
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>Smartphone GB/unidade</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C82" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="25" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="F82" s="25" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G82" s="25" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H82" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>Bernstein</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="10" t="inlineStr">
-        <is>
-          <t>Catalisadores</t>
-        </is>
-      </c>
-      <c r="B83" s="19" t="inlineStr">
-        <is>
-          <t>SK Hynix results 10-jul-26 (amanhã) · Micron FQ4 set-26 · TrendForce/UBS monthly (Fig.9 wafer adds) · Samsung prelim 2Q</t>
-        </is>
-      </c>
+          <t>UBS Fig. (BOM 12→40%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15" customHeight="1">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>H · DEBATES VIVOS, CATALISADORES E CONVENÇÕES</t>
+        </is>
+      </c>
+      <c r="B83" s="9" t="n"/>
       <c r="C83" s="9" t="n"/>
       <c r="D83" s="9" t="n"/>
       <c r="E83" s="9" t="n"/>
       <c r="F83" s="9" t="n"/>
       <c r="G83" s="9" t="n"/>
       <c r="H83" s="9" t="n"/>
-      <c r="I83" s="13" t="inlineStr">
-        <is>
-          <t>catalysts.md</t>
-        </is>
-      </c>
+      <c r="I83" s="9" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>CONVENÇÕES</t>
+          <t>Virada 2028</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
         <is>
-          <t>Gb vs GB: ÷8 · wafer HBM ≈ 1/3 dos bits de um wafer DDR (penalidade 3,1-3,5×) · servidores UBS (20,1M em 25) ≠ Gartner (12,5M) — bases distintas · GW facility ≠ GW IT-load (fora deste arquivo)</t>
+          <t>house: déficit fecha ≈0 (wafers HBM flatten ~695k, adds vão p/ DDR) vs Bernstein +5% surplus — os 109,6 bn Gb de HBM deles em 28E exigiriam ~1,1M wafers e matariam o próprio surplus</t>
         </is>
       </c>
       <c r="C84" s="9" t="n"/>
@@ -3322,40 +3445,154 @@
       <c r="H84" s="9" t="n"/>
       <c r="I84" s="13" t="inlineStr">
         <is>
+          <t>engine · Bernstein SxD</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>Alocação 26</t>
+        </is>
+      </c>
+      <c r="B85" s="19" t="inlineStr">
+        <is>
+          <t>general-server DDR ultrapassou HBM como prioridade #1 de alocação (Redburn/TrendForce) — e ainda assim HBM sobe: $17-18 → $30-32/GB 27E (Redburn) vs blended +30% (JPM/Micron)</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="n"/>
+      <c r="D85" s="9" t="n"/>
+      <c r="E85" s="9" t="n"/>
+      <c r="F85" s="9" t="n"/>
+      <c r="G85" s="9" t="n"/>
+      <c r="H85" s="9" t="n"/>
+      <c r="I85" s="13" t="inlineStr">
+        <is>
+          <t>assumptions ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B86" s="19" t="inlineStr">
+        <is>
+          <t>CXMT: 4% da oferta DRAM 25 → 12% 27E (UBS) + IPO a caminho; YMTC 41→? bn GB NAND — o wildcard de oferta pós-28</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="n"/>
+      <c r="D86" s="9" t="n"/>
+      <c r="E86" s="9" t="n"/>
+      <c r="F86" s="9" t="n"/>
+      <c r="G86" s="9" t="n"/>
+      <c r="H86" s="9" t="n"/>
+      <c r="I86" s="13" t="inlineStr">
+        <is>
+          <t>UBS · ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
+        <is>
+          <t>Conteúdo</t>
+        </is>
+      </c>
+      <c r="B87" s="19" t="inlineStr">
+        <is>
+          <t>MRDIMM 12% do mix 28E (Bernstein) + 12/16-canais → DIMMs/CPU 9→11,7 — upside de conteúdo independente de units</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="n"/>
+      <c r="D87" s="9" t="n"/>
+      <c r="E87" s="9" t="n"/>
+      <c r="F87" s="9" t="n"/>
+      <c r="G87" s="9" t="n"/>
+      <c r="H87" s="9" t="n"/>
+      <c r="I87" s="13" t="inlineStr">
+        <is>
+          <t>Bernstein</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="inlineStr">
+        <is>
+          <t>Catalisadores</t>
+        </is>
+      </c>
+      <c r="B88" s="19" t="inlineStr">
+        <is>
+          <t>SK Hynix results 10-jul-26 (amanhã) · Micron FQ4 set-26 · TrendForce/UBS monthly (Fig.9 wafer adds) · Samsung prelim 2Q</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="n"/>
+      <c r="D88" s="9" t="n"/>
+      <c r="E88" s="9" t="n"/>
+      <c r="F88" s="9" t="n"/>
+      <c r="G88" s="9" t="n"/>
+      <c r="H88" s="9" t="n"/>
+      <c r="I88" s="13" t="inlineStr">
+        <is>
+          <t>catalysts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>CONVENÇÕES</t>
+        </is>
+      </c>
+      <c r="B89" s="19" t="inlineStr">
+        <is>
+          <t>Gb vs GB: ÷8 · wafer HBM ≈ 1/3 dos bits de um wafer DDR (penalidade 3,1-3,5×) · servidores UBS (20,1M em 25) ≠ Gartner (12,5M) — bases distintas · GW facility ≠ GW IT-load (fora deste arquivo)</t>
+        </is>
+      </c>
+      <c r="C89" s="9" t="n"/>
+      <c r="D89" s="9" t="n"/>
+      <c r="E89" s="9" t="n"/>
+      <c r="F89" s="9" t="n"/>
+      <c r="G89" s="9" t="n"/>
+      <c r="H89" s="9" t="n"/>
+      <c r="I89" s="13" t="inlineStr">
+        <is>
           <t>regras da wiki</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="25">
     <mergeCell ref="B84:H84"/>
     <mergeCell ref="D2:I2"/>
     <mergeCell ref="B9:H9"/>
-    <mergeCell ref="B83:H83"/>
+    <mergeCell ref="B74:H74"/>
+    <mergeCell ref="A75:I75"/>
     <mergeCell ref="B33:H33"/>
-    <mergeCell ref="A55:I55"/>
-    <mergeCell ref="A50:I50"/>
     <mergeCell ref="A12:I12"/>
-    <mergeCell ref="B80:H80"/>
-    <mergeCell ref="B76:H76"/>
     <mergeCell ref="A26:I26"/>
+    <mergeCell ref="B89:H89"/>
+    <mergeCell ref="B85:H85"/>
     <mergeCell ref="B41:H41"/>
-    <mergeCell ref="B79:H79"/>
-    <mergeCell ref="B54:H54"/>
+    <mergeCell ref="B59:H59"/>
     <mergeCell ref="A4:I4"/>
-    <mergeCell ref="A62:I62"/>
     <mergeCell ref="B81:H81"/>
-    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="B46:H46"/>
+    <mergeCell ref="B66:H66"/>
+    <mergeCell ref="A67:I67"/>
+    <mergeCell ref="B86:H86"/>
+    <mergeCell ref="A83:I83"/>
     <mergeCell ref="A34:I34"/>
-    <mergeCell ref="B61:H61"/>
-    <mergeCell ref="B53:H53"/>
+    <mergeCell ref="B88:H88"/>
+    <mergeCell ref="A60:I60"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B82:H82"/>
-    <mergeCell ref="B69:H69"/>
-    <mergeCell ref="A70:I70"/>
-    <mergeCell ref="A78:I78"/>
+    <mergeCell ref="B87:H87"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
-  <conditionalFormatting sqref="C51:H51">
+  <conditionalFormatting sqref="C55:H55">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3363,11 +3600,27 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C52:H52">
+  <conditionalFormatting sqref="C56:H56">
     <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C57:H57">
+    <cfRule type="cellIs" priority="5" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C58:H58">
+    <cfRule type="cellIs" priority="7" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" dxfId="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
memoria auto-refresh: dashboard + resumo rebuilt from bible (18:15 task)
Automated: refresh_memoria.py after BBG/price updaters. Sources unchanged from bible.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_wiki/_dashboards/memoria-resumo.xlsx
+++ b/_wiki/_dashboards/memoria-resumo.xlsx
@@ -3808,10 +3808,10 @@
         <v>1120</v>
       </c>
       <c r="I7" t="n">
-        <v>975.5599999999999</v>
+        <v>940.4400000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>165.44</v>
+        <v>164.51</v>
       </c>
     </row>
     <row r="8">
@@ -3842,10 +3842,10 @@
         <v>728</v>
       </c>
       <c r="I8" t="n">
-        <v>2229000</v>
+        <v>1828000</v>
       </c>
       <c r="J8" t="n">
-        <v>595061.38</v>
+        <v>618346.73</v>
       </c>
     </row>
     <row r="9">
@@ -3876,10 +3876,10 @@
         <v>5969</v>
       </c>
       <c r="I9" t="n">
-        <v>290500</v>
+        <v>257500</v>
       </c>
       <c r="J9" t="n">
-        <v>67535.34</v>
+        <v>69993.14999999999</v>
       </c>
     </row>
     <row r="10">
@@ -3910,10 +3910,10 @@
         <v>540</v>
       </c>
       <c r="I10" t="n">
-        <v>76260</v>
+        <v>67100</v>
       </c>
       <c r="J10" t="n">
-        <v>12123.54</v>
+        <v>12620.8</v>
       </c>
     </row>
     <row r="11">
@@ -3944,10 +3944,10 @@
         <v>145</v>
       </c>
       <c r="I11" t="n">
-        <v>1745</v>
+        <v>1755</v>
       </c>
       <c r="J11" t="n">
-        <v>214.99</v>
+        <v>222.72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>